<commit_message>
Add numeric conversion factors to spec expressions (e.g. Al2O3+1.8895*Al)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Broken_example.xlsx
+++ b/templates/Broken_example.xlsx
@@ -684,7 +684,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>A component, or a sum of components joined with '+' (e.g. CaO+MgO). Names must match the RawMaterials headers exactly.</t>
+          <t>A component, or components joined with '+' (e.g. CaO+MgO). A component may be counted as another by a factor written before it with '*', e.g. Al2O3+1.8895*Al counts metallic Al as Al2O3 (1.8895 = 101.96 / (2 x 26.98)). Factors are numbers you type; '-' is not allowed. Names must match the RawMaterials headers exactly.</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Blank for a composition limit. Filled in (component or sum), the row limits the ratio Numerator / Denominator.</t>
+          <t>Blank for a composition limit. Filled in (same syntax as Numerator), the row limits the ratio Numerator / Denominator.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clearer spec messages, minimal conflict set, blank-cell warning, exit codes, half-up rounding; add User Guide
- Missing RawMaterials message names the --raw-materials option
- Specs: a property column or a raw material name gets its own message
- Diagnosis: the conflict set is reduced to the limits really needed
  (deletion filter); best-achievable figures kept for those that remain
- Price-range notes are printed on screen as well as in Excel
- What-if Changes: usage rows use the Recipe decimals (2 dp)
- Blank analysis cell = not analysed, 0 = analysed and absent; a warning
  when a spec uses a blank component of a material allowed in the blend
- run.py exit codes: 0 recipe found, 1 input errors, 2 no recipe
- One shared half-up rounding helper (rounding.py) for screen and Excel
- User Guide (docs/User_Guide.md, HTML and its build script)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Broken_example.xlsx
+++ b/templates/Broken_example.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -524,369 +524,381 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Type plain numbers (no units, no '&lt;0.01'). A blank component cell means 0.</t>
+          <t>Type plain numbers (no units, no '&lt;0.01').</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
+          <t>Blank or 0</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>In a component column, blank = not analysed, 0 = analysed, none present. Both count as 0, but a blank in a component that a spec uses gives a warning: type 0 if it is genuinely absent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
           <t>Analyses</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>wt %, dry basis, with LOI reported separately, so components + LOI should total 97-103 %. (Set by LAB_ANALYSIS_CONVENTION in config.py.)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="2" t="n"/>
-    </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>Sheet RawMaterials</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Unique raw material name.</t>
-        </is>
-      </c>
+      <c r="B13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Cost_Rs_per_t</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Price in Rs per tonne, on the basis given in Price_basis.</t>
+          <t>Unique raw material name.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Price_basis</t>
+          <t>Cost_Rs_per_t</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>'as_received' or 'dry'. Prices are converted to Rs per dry tonne: dry cost = cost / (1 - moisture/100) for as_received. May be blank only if moisture is 0.</t>
+          <t>Price in Rs per tonne, on the basis given in Price_basis.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Moisture_%</t>
+          <t>Price_basis</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Free moisture, wt % as received. Blank = 0.</t>
+          <t>'as_received' or 'dry'. Prices are converted to Rs per dry tonne: dry cost = cost / (1 - moisture/100) for as_received. May be blank only if moisture is 0.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>LOI_%</t>
+          <t>Moisture_%</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Loss on ignition, wt % dry basis. Blank = 0.</t>
+          <t>Free moisture, wt % as received. Blank = 0.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Min_use_%</t>
+          <t>LOI_%</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Plant-wide minimum use, wt % of the dry blend. Blank = 0.</t>
+          <t>Loss on ignition, wt % dry basis. Blank = 0.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Max_use_%</t>
+          <t>Min_use_%</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Plant-wide maximum use, wt % of the dry blend. Blank = 100.</t>
+          <t>Plant-wide minimum use, wt % of the dry blend. Blank = 0.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>Max_use_%</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Plant-wide maximum use, wt % of the dry blend. Blank = 100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>Any other column</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>A chemical component, wt % (see 'Analyses' above). Add, remove or reorder component columns freely; the header is the component name.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="n"/>
-      <c r="B21" s="2" t="n"/>
-    </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Sheet Specs</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>One row per limit.</t>
-        </is>
-      </c>
+      <c r="A22" s="3" t="n"/>
+      <c r="B22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Sheet Specs</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Unique label. The constraints are named &lt;Name&gt;_min and &lt;Name&gt;_max in the report.</t>
+          <t>One row per limit.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Numerator</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>A component, or components joined with '+' (e.g. CaO+MgO). A component may be counted as another by a factor written before it with '*', e.g. Al2O3+1.8895*Al counts metallic Al as Al2O3 (1.8895 = 101.96 / (2 x 26.98)). Factors are numbers you type; '-' is not allowed. Names must match the RawMaterials headers exactly.</t>
+          <t>Unique label. The constraints are named &lt;Name&gt;_min and &lt;Name&gt;_max in the report.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Denominator</t>
+          <t>Numerator</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Blank for a composition limit. Filled in (same syntax as Numerator), the row limits the ratio Numerator / Denominator.</t>
+          <t>A component, or components joined with '+' (e.g. CaO+MgO). A component may be counted as another by a factor written before it with '*', e.g. Al2O3+1.8895*Al counts metallic Al as Al2O3 (1.8895 = 101.96 / (2 x 26.98)). Factors are numbers you type; '-' is not allowed. Names must match the RawMaterials headers exactly.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Min, Max</t>
+          <t>Denominator</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>The customer limits. Blank = no limit; at least one is needed.</t>
+          <t>Blank for a composition limit. Filled in (same syntax as Numerator), the row limits the ratio Numerator / Denominator.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
+          <t>Min, Max</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>The customer limits. Blank = no limit; at least one is needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
           <t>Margin</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Safety margin in the same unit as Min/Max, applied inward (target = Min + margin, Max - margin). Blank = 0.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="n"/>
-      <c r="B28" s="2" t="n"/>
-    </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>Sheet Settings</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Two columns, Key and Value.</t>
-        </is>
-      </c>
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Product_name</t>
+          <t>Sheet Settings</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Shown in the report.</t>
+          <t>Two columns, Key and Value.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Spec_basis</t>
+          <t>Product_name</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Basis of the composition limits: dry, as_received, ignited (default dry). Ratio limits do not depend on it.</t>
+          <t>Shown in the report.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Batch_size_kg</t>
+          <t>Spec_basis</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Total as-received mass weighed into the mixer, kg (default 1000).</t>
+          <t>Basis of the composition limits: dry, as_received, ignited (default dry). Ratio limits do not depend on it.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
+          <t>Batch_size_kg</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Total as-received mass weighed into the mixer, kg (default 1000).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
           <t>Scale_resolution_kg</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Optional. Resolution of the weighing scale, kg; the weigh sheet is rounded to it. Blank = 0.1 (config.py).</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="3" t="n"/>
-      <c r="B34" s="2" t="n"/>
-    </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>Sheet UsageLimits (optional)</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Product- or customer-specific usage limits.</t>
-        </is>
-      </c>
+      <c r="A35" s="3" t="n"/>
+      <c r="B35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Sheet UsageLimits (optional)</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Must match a name in RawMaterials.</t>
+          <t>Product- or customer-specific usage limits.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Must match a name in RawMaterials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
           <t>Min_use_%, Max_use_%</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>wt % of the dry blend. The tighter of these and the plant-wide limits applies. Max 0 bans a material.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="3" t="n"/>
-      <c r="B38" s="2" t="n"/>
-    </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>Sheet WhatIf (optional)</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>What-if scenarios, each compared with the base case. One row per change; rows with the same Scenario name form one scenario.</t>
-        </is>
-      </c>
+      <c r="A39" s="3" t="n"/>
+      <c r="B39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Scenario</t>
+          <t>Sheet WhatIf (optional)</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Any name, e.g. 'Fluorspar dearer'.</t>
+          <t>What-if scenarios, each compared with the base case. One row per change; rows with the same Scenario name form one scenario.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Change type</t>
+          <t>Scenario</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Price (Item = raw material, value = Rs/t in its own price basis); Spec Min / Spec Max / Spec Margin (Item = spec Name; blank Min/Max removes that limit, blank Margin = 0); Usage Min / Usage Max (Item = raw material, value = wt % of dry blend; replaces its UsageLimits value, the plant-wide limit still applies).</t>
+          <t>Any name, e.g. 'Fluorspar dearer'.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Change type</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>The raw material or spec Name being changed.</t>
+          <t>Price (Item = raw material, value = Rs/t in its own price basis); Spec Min / Spec Max / Spec Margin (Item = spec Name; blank Min/Max removes that limit, blank Margin = 0); Usage Min / Usage Max (Item = raw material, value = wt % of dry blend; replaces its UsageLimits value, the plant-wide limit still applies).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>The raw material or spec Name being changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
           <t>New value</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>The new value (see Change type).</t>
         </is>

</xml_diff>